<commit_message>
ACH.Operator seed / usuario operador sintético
</commit_message>
<xml_diff>
--- a/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
+++ b/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
@@ -501,7 +501,7 @@
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="35" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
@@ -581,17 +581,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19 09:47</t>
+          <t>2026-05-19 10:46</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>ACH-Interbank-Postgresql</t>
+          <t>fix/uat-operator-role-seed</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>7a94a633</t>
+          <t>efac77e4</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>67.6 / 100</t>
+          <t>67.8 / 100</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -647,8 +647,8 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="36" customWidth="1" min="11" max="11"/>
   </cols>
@@ -878,15 +878,19 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Captura pantalla</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr"/>
+          <t>Captura pantalla/login sanitizado</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Login/JWT evidencia Admin y ACH.Operator</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
           <t>DEF-UAT-015</t>
@@ -894,7 +898,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>ACH.Operator pendiente.</t>
+          <t>Cerrado para UAT controlado.</t>
         </is>
       </c>
     </row>
@@ -1783,18 +1787,18 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="41" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
     <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="35" customWidth="1" min="15" max="15"/>
+    <col width="45" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2941,22 +2945,22 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Validar rol operador si se corrige seed.</t>
+          <t>Validar rol operador con usuario demo multirol.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>ACH.Operator</t>
+          <t>Admin + ACH.Operator</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Seed corregido o usuario operador</t>
+          <t>Seed/migracion aplicada</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Usuario sintetico</t>
+          <t>Usuario demo admin sin password documentado</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -2969,13 +2973,21 @@
           <t>Rol visible y autorizado.</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Admin y ACH.Operator visibles en respuesta/JWT sanitizados.</t>
+        </is>
+      </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr"/>
+          <t>Ejecutada OK</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>EV-FUNC-039</t>
+        </is>
+      </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
           <t>DEF-UAT-015</t>
@@ -2988,7 +3000,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Pendiente por brecha.</t>
+          <t>Cerrado para UAT controlado; evaluar usuario operador separado antes de productivo.</t>
         </is>
       </c>
     </row>
@@ -4115,13 +4127,13 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4212,7 +4224,11 @@
           <t>ACH.Operator no asignado/no visible.</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>EV-FUNC-039</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Seguridad/Backend</t>
@@ -4220,17 +4236,29 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Abierto</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
+          <t>Opcion A: admin demo multirol para UAT controlado</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>No debilita auth; evaluar operador separado para productivo.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4908,7 +4936,7 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5276,7 +5304,11 @@
           <t>Seguridad</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>ACH.Operator cerrado para UAT; siguen secretos/certificados/OpenBao segun alcance.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
UAT funcional nacha-m y Proc_Contrapartidas
</commit_message>
<xml_diff>
--- a/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
+++ b/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
@@ -19,11 +19,11 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$1:$K$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checklist_UAT_Operativo'!$A$1:$K$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Set_Pruebas_Operativas'!$A$1:$O$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Set_Pruebas_Operativas'!$A$1:$O$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Evidencias'!$A$1:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Defectos'!$A$1:$L$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Defectos'!$A$1:$L$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Datos_Sinteticos'!$A$1:$G$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Criterios_GO_NO_GO'!$A$1:$G$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Criterios_GO_NO_GO'!$A$1:$G$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Firmas_Aprobaciones'!$A$1:$G$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -501,7 +501,7 @@
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="35" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
@@ -581,17 +581,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19 10:46</t>
+          <t>2026-05-19 11:53</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>fix/uat-operator-role-seed</t>
+          <t>uat/nacha-m-soap-proc-contrapartidas</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>efac77e4</t>
+          <t>98934e01</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>67.8 / 100</t>
+          <t>67.4 / 100</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -1781,21 +1781,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="41" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="45" customWidth="1" min="15" max="15"/>
@@ -3053,7 +3053,7 @@
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Bloqueada</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr"/>
@@ -3067,7 +3067,11 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>UAT integrado 2026-05-19 no obtuvo archivo NACHA-M valido.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3792,8 +3796,146 @@
       </c>
       <c r="O31" s="2" t="inlineStr"/>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>UAT-OP-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>NACHA-M</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Validar archivo NACHA-M no vacio por camara</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Confirmar que ACH Colombia y CENIT generan archivo real UAT por sistema.</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Admin/QA</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Transacciones exportables y prenotificacion previa cumplida</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Datos sinteticos</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Generar por /NachaExport o nacha-security y revisar size/hash/registros.</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Archivo &gt; 0 bytes, no HTML/JSON error, registros 1/5/6/8/9.</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Bloqueada</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>docs/uat/evidencias/nacha-m-uat/</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>DEF-UAT-021</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>UAT-OP-032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>SOAP</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Validar Proc_Contrapartidas dry-run/mock</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Confirmar que el job SOAP no usa endpoint externo no autorizado.</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Admin/Integracion</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Endpoint UAT/mock o dry-run configurado</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Payload sintetico</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Ejecutar dry-run autorizado y revisar request/response sanitizado.</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Sin transmision productiva; XML bien formado y auditado.</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Bloqueada</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>docs/uat/evidencias/soap-proc-contrapartidas/</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>DEF-UAT-022</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O31"/>
+  <autoFilter ref="A1:O33"/>
   <conditionalFormatting sqref="K2:K500">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
@@ -4119,7 +4261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4127,8 +4269,8 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -4283,10 +4425,14 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>NACHA-M 1/5/6/7/8/9 pendiente campo-a-campo.</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
+          <t>NACHA-M 1/5/6/7/8/9 pendiente campo-a-campo; UAT integrado no genero archivo valido.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>docs/uat/EVIDENCIAS_NACHA_M_UAT.md</t>
+        </is>
+      </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Arquitectura ACH/QA</t>
@@ -4297,45 +4443,57 @@
           <t>Abierto</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Requiere archivo no vacio, matriz y homologacion/waiver.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CENIT-CUD</t>
+          <t>DEF-UAT-021</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>UAT-OP-027</t>
+          <t>UAT-OP-031</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>CENIT</t>
+          <t>NACHA-M</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Bloqueante</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>CENIT/CUD pendiente.</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
+          <t>/NachaExport devuelve 200 con archivo vacio en escenario no exportable.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>docs/uat/evidencias/nacha-m-uat/</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Integracion/Negocio</t>
+          <t>Backend/QA</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -4343,45 +4501,57 @@
           <t>Abierto</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Debe retornar error controlado o archivo valido.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>SOBRE-DIGITAL</t>
+          <t>DEF-UAT-022</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>UAT-OP-028</t>
+          <t>UAT-OP-032</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>SOAP</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Bloqueante</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sobre digital/firma/certificados pendiente.</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr"/>
+          <t>Proc_Contrapartidas requiere UAT/mock o guardrail dry-run; job intento endpoint externo no resoluble.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>docs/uat/EVIDENCIAS_SOAP_PROC_CONTRAPARTIDAS.md</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Seguridad/Integracion</t>
+          <t>Integracion/DevOps/Seguridad</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -4389,29 +4559,37 @@
           <t>Abierto</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>No hubo transmision exitosa.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>BKP-RESTORE</t>
+          <t>CENIT-CUD</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>UAT-OP-029</t>
+          <t>UAT-OP-027</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Operacion</t>
+          <t>CENIT</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -4421,13 +4599,13 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Backup/restore/rollback pendiente.</t>
+          <t>CENIT/CUD pendiente.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Operaciones/SRE</t>
+          <t>Integracion/Negocio</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -4444,8 +4622,100 @@
       </c>
       <c r="L6" s="2" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SOBRE-DIGITAL</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>UAT-OP-028</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Bloqueante</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Sobre digital/firma/certificados pendiente.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Seguridad/Integracion</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>BKP-RESTORE</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>UAT-OP-029</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Operacion</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Bloqueante</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Backup/restore/rollback pendiente.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Operaciones/SRE</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L6"/>
+  <autoFilter ref="A1:L8"/>
   <conditionalFormatting sqref="H2:H500">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
@@ -4927,15 +5197,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -5149,12 +5419,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>BLOQUEADO</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Matriz NACHA-M</t>
+          <t>Matriz NACHA-M / evidencias 0 bytes</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -5164,7 +5434,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Registros 1/5/6/7/8/9 validados</t>
+          <t>Registros 1/5/6/7/8/9 validados con archivo no vacio</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -5172,22 +5442,26 @@
           <t>Arquitectura ACH</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Resolver DEF-UAT-020/021.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CENIT/CUD</t>
+          <t>Proc_Contrapartidas dry-run/mock</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Brechas</t>
+          <t>Envelopes XML sanitizados</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -5197,20 +5471,24 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Validacion o waiver</t>
+          <t>Endpoint UAT/mock o dry-run con no transmision</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Integracion</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
+          <t>Integracion/DevOps</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Resolver DEF-UAT-022.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Sobre digital</t>
+          <t>CENIT/CUD</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -5230,12 +5508,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Firma/certificados validados</t>
+          <t>Validacion o waiver</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Integracion</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -5243,7 +5521,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Certificados</t>
+          <t>Sobre digital</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -5253,7 +5531,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Revision seguridad</t>
+          <t>Brechas</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -5263,7 +5541,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Certificados de prueba y custodia aprobada</t>
+          <t>Firma/certificados validados</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -5276,54 +5554,50 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>Certificados</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Revision seguridad</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Certificados de prueba y custodia aprobada</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>Seguridad</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Revision seguridad</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Brechas cerradas o aceptadas formalmente</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Seguridad</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>ACH.Operator cerrado para UAT; siguen secretos/certificados/OpenBao segun alcance.</t>
-        </is>
-      </c>
+      <c r="G11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>OpenBao/secrets</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Brechas</t>
+          <t>Revision seguridad</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -5333,20 +5607,24 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Gestion de secretos validada</t>
+          <t>Brechas cerradas o aceptadas formalmente</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>DevOps/Security</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>ACH.Operator cerrado para UAT; siguen secretos/certificados/OpenBao segun alcance.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Backup/restore</t>
+          <t>OpenBao/secrets</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -5366,12 +5644,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Prueba aprobada</t>
+          <t>Gestion de secretos validada</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>DevOps/Security</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -5379,7 +5657,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Actas</t>
+          <t>Backup/restore</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -5389,7 +5667,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Actas UAT</t>
+          <t>Brechas</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -5399,12 +5677,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Firmas completas</t>
+          <t>Prueba aprobada</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>PMO/QA</t>
+          <t>SRE</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
@@ -5412,42 +5690,75 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>Actas</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Actas UAT</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Firmas completas</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>PMO/QA</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>Aprobaciones</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Comite</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Si</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Aprobaciones formales</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Direccion</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Productivo: NO-GO.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G15"/>
+  <autoFilter ref="A1:G16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Cerré técnicamente DEF-UAT-021 y DEF-UAT-022 para UAT/local
</commit_message>
<xml_diff>
--- a/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
+++ b/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19 11:53</t>
+          <t>2026-05-19 13:06</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>98934e01</t>
+          <t>f8c39d53</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>67.4 / 100</t>
+          <t>68.1 / 100</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -3842,7 +3842,11 @@
           <t>Archivo &gt; 0 bytes, no HTML/JSON error, registros 1/5/6/8/9.</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Bloqueado por prenotificacion previa ausente; /NachaExport retorna 422 JSON controlado.</t>
+        </is>
+      </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
           <t>Bloqueada</t>
@@ -3855,7 +3859,7 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>DEF-UAT-021</t>
+          <t>DEF-UAT-020</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
@@ -3863,7 +3867,11 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="O32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>DEF-UAT-021 cerrado tecnicamente; falta archivo no vacio con prenotificacion valida.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3911,15 +3919,19 @@
           <t>Sin transmision productiva; XML bien formado y auditado.</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>DryRun runtime validado con PROC_DRY_RUN sin invocacion SOAP externa.</t>
+        </is>
+      </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Ejecutada OK</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>docs/uat/evidencias/soap-proc-contrapartidas/</t>
+          <t>docs/uat/evidencias/soap-proc-contrapartidas/runtime_dry_run_validation.md</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
@@ -3932,7 +3944,11 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="O33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>Cerrado tecnico UAT/local; endpoint UAT/mock real pendiente para homologacion.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O33"/>
@@ -4483,12 +4499,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>/NachaExport devuelve 200 con archivo vacio en escenario no exportable.</t>
+          <t>/NachaExport ya no devuelve 200 con archivo vacio; responde 422 JSON controlado cuando faltan prerequisitos/exportables.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>docs/uat/evidencias/nacha-m-uat/</t>
+          <t>docs/uat/evidencias/nacha-m-uat/*/attempt_4_controlled_422_response.txt</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -4498,7 +4514,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -4506,15 +4522,19 @@
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Cerrado tecnico</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Debe retornar error controlado o archivo valido.</t>
+          <t>Pendiente reintento con prenotificacion valida para cerrar DEF-UAT-020.</t>
         </is>
       </c>
     </row>
@@ -4541,12 +4561,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Proc_Contrapartidas requiere UAT/mock o guardrail dry-run; job intento endpoint externo no resoluble.</t>
+          <t>Proc_Contrapartidas queda protegido por DryRun en UAT/local; no invoca endpoint externo sin modo Live explicito.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>docs/uat/EVIDENCIAS_SOAP_PROC_CONTRAPARTIDAS.md</t>
+          <t>docs/uat/evidencias/soap-proc-contrapartidas/runtime_dry_run_validation.md</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -4556,7 +4576,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -4564,15 +4584,19 @@
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Cerrado tecnico UAT/local</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>No hubo transmision exitosa.</t>
+          <t>Endpoint UAT/mock real pendiente para homologacion; Productivo NO-GO.</t>
         </is>
       </c>
     </row>
@@ -4770,12 +4794,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5008,17 +5032,17 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Banco origen</t>
+          <t>Banco origen default</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Banco UAT Origen</t>
+          <t>Cooperativa Financiera de Antioquia (CFA default source)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Datos maestros sinteticos</t>
+          <t>Datos maestros UAT/default</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -5033,7 +5057,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>No banco productivo real.</t>
+          <t>Unica institucion IsDefaultSource=true; Banco UAT Origen no es default.</t>
         </is>
       </c>
     </row>
@@ -5202,7 +5226,7 @@
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="37" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
@@ -5424,7 +5448,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Matriz NACHA-M / evidencias 0 bytes</t>
+          <t>422 JSON controlado por prenotificacion previa ausente; sin archivo no vacio</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -5444,7 +5468,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Resolver DEF-UAT-020/021.</t>
+          <t>Resolver DEF-UAT-020 con prenotificacion UAT valida; DEF-UAT-021 cerrado tecnico.</t>
         </is>
       </c>
     </row>
@@ -5456,12 +5480,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>OK UAT/LOCAL</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Envelopes XML sanitizados</t>
+          <t>runtime_dry_run_validation.md</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -5471,7 +5495,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Endpoint UAT/mock o dry-run con no transmision</t>
+          <t>Endpoint UAT/mock homologado o Live aprobado formalmente</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -5481,7 +5505,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Resolver DEF-UAT-022.</t>
+          <t>DEF-UAT-022 cerrado tecnico UAT/local; Productivo NO-GO.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
generaron archivos NACHA-M UAT no vacíos por ACH
</commit_message>
<xml_diff>
--- a/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
+++ b/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19 22:16</t>
+          <t>2026-05-19 23:35</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>03607c24</t>
+          <t>48759d45</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
UAT controlado de prenotificaciones CFA
</commit_message>
<xml_diff>
--- a/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
+++ b/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20 11:03</t>
+          <t>2026-05-20 12:28</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>ffe311cf</t>
+          <t>33bbc145</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Simulador NACHA-M de Entrada para UAT/local
</commit_message>
<xml_diff>
--- a/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
+++ b/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20 12:28</t>
+          <t>2026-05-20 15:52</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>33bbc145</t>
+          <t>80ac77b8</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
paquete final UAT SOAP end-to-end con acta firmable
</commit_message>
<xml_diff>
--- a/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
+++ b/docs/comite-go-no-go/exports/Excel/CHECKLIST_UAT_OPERATIVO_ACH_INTERBANK.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20 15:52</t>
+          <t>2026-05-23 19:03</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>80ac77b8</t>
+          <t>cdd126cf</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">

</xml_diff>